<commit_message>
Major update: 14 alarms classified
</commit_message>
<xml_diff>
--- a/AlarmOntoClassification.xlsx
+++ b/AlarmOntoClassification.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rzoodsm2/Documents/GIT-repositories/Alarm-Ontologie/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDBC3F44-F5BC-4D40-898A-9437465E0D23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DB9306C-D38E-A74C-8633-90633ADC5D95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="18360" xr2:uid="{CBFFA7CC-2A3B-794A-9F55-02AECC0222F5}"/>
+    <workbookView xWindow="4740" yWindow="620" windowWidth="38400" windowHeight="21100" activeTab="3" xr2:uid="{CBFFA7CC-2A3B-794A-9F55-02AECC0222F5}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
     <sheet name="Blad2" sheetId="2" r:id="rId2"/>
     <sheet name="Analyse_Subset" sheetId="3" r:id="rId3"/>
+    <sheet name="Blad3" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -60,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7159" uniqueCount="945">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7442" uniqueCount="992">
   <si>
     <t>CRITICOOL - Verbinding verbroken</t>
   </si>
@@ -2895,6 +2896,147 @@
   </si>
   <si>
     <t>Patient_X</t>
+  </si>
+  <si>
+    <t>Integumentary, Cardiovascular, Endocrine, Nervous</t>
+  </si>
+  <si>
+    <t>Pulmonary_diffusion, Pulmonary_Ventilation</t>
+  </si>
+  <si>
+    <t>ArterialOxygenation</t>
+  </si>
+  <si>
+    <t>CardiacElectricalDepolarization</t>
+  </si>
+  <si>
+    <t>Skin_temperature</t>
+  </si>
+  <si>
+    <t>Core_temperature</t>
+  </si>
+  <si>
+    <t>Cardiac_Contractile_rate</t>
+  </si>
+  <si>
+    <t>ArterialBloodPressure</t>
+  </si>
+  <si>
+    <t>ArterialCarbonDioxide</t>
+  </si>
+  <si>
+    <t>ECGModule</t>
+  </si>
+  <si>
+    <t>TempModule</t>
+  </si>
+  <si>
+    <t>BatteryModule</t>
+  </si>
+  <si>
+    <t>IBP_Module</t>
+  </si>
+  <si>
+    <t>Capnography_Module</t>
+  </si>
+  <si>
+    <t>ST-II</t>
+  </si>
+  <si>
+    <t>ST-V</t>
+  </si>
+  <si>
+    <t>Temp_Skin</t>
+  </si>
+  <si>
+    <t>Temp_Core</t>
+  </si>
+  <si>
+    <t>PulsatileHeartRate</t>
+  </si>
+  <si>
+    <t>ArterialBP</t>
+  </si>
+  <si>
+    <t>EtCO2</t>
+  </si>
+  <si>
+    <t>SpO2_Channel</t>
+  </si>
+  <si>
+    <t>SkinTemp_Channel</t>
+  </si>
+  <si>
+    <t>CoreTemp_channel</t>
+  </si>
+  <si>
+    <t>ST_II_Channel</t>
+  </si>
+  <si>
+    <t>ST_V_Channel</t>
+  </si>
+  <si>
+    <t>PulseRate_Channel</t>
+  </si>
+  <si>
+    <t>EtCO2_Channel</t>
+  </si>
+  <si>
+    <t>ABP_channel</t>
+  </si>
+  <si>
+    <t>PulseOx_Waveform</t>
+  </si>
+  <si>
+    <t>Capno_Waveform</t>
+  </si>
+  <si>
+    <t>ABP_Waveform</t>
+  </si>
+  <si>
+    <t>PulseOximeter</t>
+  </si>
+  <si>
+    <t>ECG</t>
+  </si>
+  <si>
+    <t>SkinTempSensor</t>
+  </si>
+  <si>
+    <t>CoreTempSensor</t>
+  </si>
+  <si>
+    <t>PulseOx_Interface</t>
+  </si>
+  <si>
+    <t>ECG_Interface</t>
+  </si>
+  <si>
+    <t>Temp_Interface</t>
+  </si>
+  <si>
+    <t>BP_transducer_interface</t>
+  </si>
+  <si>
+    <t>CO2_Sensor_interface</t>
+  </si>
+  <si>
+    <t>Endocrine</t>
+  </si>
+  <si>
+    <t>Nervous</t>
+  </si>
+  <si>
+    <t>Pulmonary_Diffusion</t>
+  </si>
+  <si>
+    <t>PulseOx_Waveform_Analysis</t>
+  </si>
+  <si>
+    <t>ECG_Waveform_analysis</t>
+  </si>
+  <si>
+    <t>Capno_Waveform_Analysis</t>
   </si>
 </sst>
 </file>
@@ -3091,7 +3233,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -3121,6 +3263,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" textRotation="125"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment textRotation="135" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3131,9 +3277,14 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment textRotation="135" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -3489,24 +3640,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="22" x14ac:dyDescent="0.3">
-      <c r="N1" s="25" t="s">
+      <c r="N1" s="27" t="s">
         <v>571</v>
       </c>
-      <c r="O1" s="26"/>
-      <c r="P1" s="26"/>
-      <c r="Q1" s="26"/>
-      <c r="R1" s="26"/>
-      <c r="S1" s="27"/>
-      <c r="T1" s="25" t="s">
+      <c r="O1" s="28"/>
+      <c r="P1" s="28"/>
+      <c r="Q1" s="28"/>
+      <c r="R1" s="28"/>
+      <c r="S1" s="29"/>
+      <c r="T1" s="27" t="s">
         <v>572</v>
       </c>
-      <c r="U1" s="26"/>
-      <c r="V1" s="26"/>
-      <c r="W1" s="26"/>
-      <c r="X1" s="26"/>
-      <c r="Y1" s="26"/>
-      <c r="Z1" s="26"/>
-      <c r="AA1" s="27"/>
+      <c r="U1" s="28"/>
+      <c r="V1" s="28"/>
+      <c r="W1" s="28"/>
+      <c r="X1" s="28"/>
+      <c r="Y1" s="28"/>
+      <c r="Z1" s="28"/>
+      <c r="AA1" s="29"/>
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -33626,7 +33777,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66A7E2AF-4348-274C-8FED-9C3AA44A5E7F}">
-  <dimension ref="B1:AU79"/>
+  <dimension ref="C1:AU79"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.6640625" bestFit="1" customWidth="1"/>
@@ -33650,127 +33801,127 @@
       <c r="F1" s="6" t="s">
         <v>943</v>
       </c>
-      <c r="G1" s="28" t="s">
+      <c r="G1" s="25" t="s">
         <v>197</v>
       </c>
-      <c r="H1" s="28" t="s">
+      <c r="H1" s="25" t="s">
         <v>200</v>
       </c>
-      <c r="I1" s="28" t="s">
+      <c r="I1" s="25" t="s">
         <v>201</v>
       </c>
-      <c r="J1" s="28" t="s">
+      <c r="J1" s="25" t="s">
         <v>202</v>
       </c>
-      <c r="K1" s="28" t="s">
+      <c r="K1" s="25" t="s">
         <v>203</v>
       </c>
-      <c r="L1" s="28" t="s">
+      <c r="L1" s="25" t="s">
         <v>204</v>
       </c>
-      <c r="M1" s="28" t="s">
+      <c r="M1" s="25" t="s">
         <v>205</v>
       </c>
-      <c r="N1" s="28" t="s">
+      <c r="N1" s="25" t="s">
         <v>207</v>
       </c>
-      <c r="O1" s="28" t="s">
+      <c r="O1" s="25" t="s">
         <v>208</v>
       </c>
-      <c r="P1" s="28" t="s">
+      <c r="P1" s="25" t="s">
         <v>209</v>
       </c>
-      <c r="Q1" s="28" t="s">
+      <c r="Q1" s="25" t="s">
         <v>211</v>
       </c>
-      <c r="R1" s="28" t="s">
+      <c r="R1" s="25" t="s">
         <v>213</v>
       </c>
-      <c r="S1" s="28" t="s">
+      <c r="S1" s="25" t="s">
         <v>215</v>
       </c>
-      <c r="T1" s="28" t="s">
+      <c r="T1" s="25" t="s">
         <v>217</v>
       </c>
-      <c r="U1" s="28" t="s">
+      <c r="U1" s="25" t="s">
         <v>220</v>
       </c>
-      <c r="V1" s="28" t="s">
+      <c r="V1" s="25" t="s">
         <v>223</v>
       </c>
-      <c r="W1" s="28" t="s">
+      <c r="W1" s="25" t="s">
         <v>235</v>
       </c>
-      <c r="X1" s="28" t="s">
+      <c r="X1" s="25" t="s">
         <v>242</v>
       </c>
-      <c r="Y1" s="28" t="s">
+      <c r="Y1" s="25" t="s">
         <v>246</v>
       </c>
-      <c r="Z1" s="28" t="s">
+      <c r="Z1" s="25" t="s">
         <v>247</v>
       </c>
-      <c r="AA1" s="28" t="s">
+      <c r="AA1" s="25" t="s">
         <v>264</v>
       </c>
-      <c r="AB1" s="28" t="s">
+      <c r="AB1" s="25" t="s">
         <v>266</v>
       </c>
-      <c r="AC1" s="28" t="s">
+      <c r="AC1" s="25" t="s">
         <v>292</v>
       </c>
-      <c r="AD1" s="28" t="s">
+      <c r="AD1" s="25" t="s">
         <v>293</v>
       </c>
-      <c r="AE1" s="28" t="s">
+      <c r="AE1" s="25" t="s">
         <v>377</v>
       </c>
-      <c r="AF1" s="28" t="s">
+      <c r="AF1" s="25" t="s">
         <v>378</v>
       </c>
-      <c r="AG1" s="28" t="s">
+      <c r="AG1" s="25" t="s">
         <v>417</v>
       </c>
-      <c r="AH1" s="28" t="s">
+      <c r="AH1" s="25" t="s">
         <v>418</v>
       </c>
-      <c r="AI1" s="28" t="s">
+      <c r="AI1" s="25" t="s">
         <v>314</v>
       </c>
-      <c r="AJ1" s="28" t="s">
+      <c r="AJ1" s="25" t="s">
         <v>501</v>
       </c>
-      <c r="AK1" s="28" t="s">
+      <c r="AK1" s="25" t="s">
         <v>502</v>
       </c>
-      <c r="AL1" s="28" t="s">
+      <c r="AL1" s="25" t="s">
         <v>526</v>
       </c>
-      <c r="AM1" s="28" t="s">
+      <c r="AM1" s="25" t="s">
         <v>533</v>
       </c>
-      <c r="AN1" s="28" t="s">
+      <c r="AN1" s="25" t="s">
         <v>550</v>
       </c>
-      <c r="AO1" s="28" t="s">
+      <c r="AO1" s="25" t="s">
         <v>546</v>
       </c>
-      <c r="AP1" s="28" t="s">
+      <c r="AP1" s="25" t="s">
         <v>554</v>
       </c>
-      <c r="AQ1" s="28" t="s">
+      <c r="AQ1" s="25" t="s">
         <v>556</v>
       </c>
-      <c r="AR1" s="28" t="s">
+      <c r="AR1" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="AS1" s="28" t="s">
+      <c r="AS1" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="AT1" s="28" t="s">
+      <c r="AT1" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="AU1" s="28" t="s">
+      <c r="AU1" s="25" t="s">
         <v>67</v>
       </c>
     </row>
@@ -33887,7 +34038,7 @@
       <c r="AE3" s="5"/>
       <c r="AF3" s="5"/>
       <c r="AG3" s="5" t="str">
-        <f t="shared" ref="AG3:AH3" si="2">AG6</f>
+        <f t="shared" ref="AG3" si="2">AG6</f>
         <v>Pulmonary</v>
       </c>
       <c r="AH3" s="5"/>
@@ -34143,7 +34294,7 @@
       <c r="AE7" s="5"/>
       <c r="AF7" s="5"/>
       <c r="AG7" s="5" t="str">
-        <f t="shared" ref="AG7:AH7" si="5">AG11</f>
+        <f t="shared" ref="AG7" si="5">AG11</f>
         <v>Lungs</v>
       </c>
       <c r="AH7" s="5"/>
@@ -34449,7 +34600,7 @@
       <c r="AE12" s="5"/>
       <c r="AF12" s="5"/>
       <c r="AG12" s="5" t="str">
-        <f t="shared" ref="AG12:AH12" si="8">AG16</f>
+        <f t="shared" ref="AG12" si="8">AG16</f>
         <v>Pulmonary_Oxygenation</v>
       </c>
       <c r="AH12" s="5"/>
@@ -35105,7 +35256,7 @@
       <c r="AE23" s="5"/>
       <c r="AF23" s="5"/>
       <c r="AG23" s="5" t="str">
-        <f t="shared" ref="AG23:AH23" si="14">AG16</f>
+        <f t="shared" ref="AG23" si="14">AG16</f>
         <v>Pulmonary_Oxygenation</v>
       </c>
       <c r="AH23" s="5" t="s">
@@ -37202,7 +37353,7 @@
       <c r="O56" s="13" t="s">
         <v>826</v>
       </c>
-      <c r="P56" s="29" t="s">
+      <c r="P56" s="26" t="s">
         <v>845</v>
       </c>
       <c r="Q56" s="13" t="s">
@@ -38804,5 +38955,943 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4409A81-4142-C744-BB80-FD175F01C181}">
+  <dimension ref="A1:AF28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="29.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.1640625" customWidth="1"/>
+    <col min="4" max="4" width="22.1640625" customWidth="1"/>
+    <col min="5" max="5" width="15.1640625" customWidth="1"/>
+    <col min="8" max="8" width="19.6640625" customWidth="1"/>
+    <col min="9" max="9" width="17.6640625" customWidth="1"/>
+    <col min="11" max="11" width="25.83203125" customWidth="1"/>
+    <col min="12" max="12" width="20.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:32" ht="194" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B1" s="25" t="s">
+        <v>197</v>
+      </c>
+      <c r="C1" s="25" t="s">
+        <v>200</v>
+      </c>
+      <c r="D1" s="25" t="s">
+        <v>205</v>
+      </c>
+      <c r="E1" s="25" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1" s="25" t="s">
+        <v>213</v>
+      </c>
+      <c r="G1" s="25" t="s">
+        <v>215</v>
+      </c>
+      <c r="H1" s="25" t="s">
+        <v>220</v>
+      </c>
+      <c r="I1" s="25" t="s">
+        <v>242</v>
+      </c>
+      <c r="J1" s="25" t="s">
+        <v>247</v>
+      </c>
+      <c r="K1" s="25" t="s">
+        <v>266</v>
+      </c>
+      <c r="L1" s="25" t="s">
+        <v>377</v>
+      </c>
+      <c r="M1" s="25" t="s">
+        <v>378</v>
+      </c>
+      <c r="N1" s="25" t="s">
+        <v>417</v>
+      </c>
+      <c r="O1" s="25" t="s">
+        <v>314</v>
+      </c>
+      <c r="P1" s="25"/>
+      <c r="Q1" s="25"/>
+      <c r="R1" s="25"/>
+      <c r="S1" s="25"/>
+      <c r="T1" s="25"/>
+      <c r="U1" s="25"/>
+      <c r="V1" s="25"/>
+      <c r="W1" s="25"/>
+      <c r="X1" s="25"/>
+      <c r="Y1" s="25"/>
+      <c r="Z1" s="25"/>
+      <c r="AA1" s="25"/>
+      <c r="AB1" s="25"/>
+      <c r="AC1" s="25"/>
+      <c r="AD1" s="25"/>
+      <c r="AE1" s="25"/>
+      <c r="AF1" s="25"/>
+    </row>
+    <row r="3" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>573</v>
+      </c>
+      <c r="B3" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="C3" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="D3" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="E3" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="F3" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="G3" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="H3" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="I3" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="J3" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="K3" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="L3" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="M3" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="N3" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="O3" s="30" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="4" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>574</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>586</v>
+      </c>
+      <c r="E4" t="s">
+        <v>586</v>
+      </c>
+      <c r="F4" t="s">
+        <v>945</v>
+      </c>
+      <c r="G4" t="s">
+        <v>945</v>
+      </c>
+      <c r="H4" t="s">
+        <v>586</v>
+      </c>
+      <c r="I4" t="s">
+        <v>586</v>
+      </c>
+      <c r="J4" t="s">
+        <v>586</v>
+      </c>
+      <c r="K4" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="L4" t="s">
+        <v>586</v>
+      </c>
+      <c r="M4" t="s">
+        <v>586</v>
+      </c>
+      <c r="N4" t="s">
+        <v>12</v>
+      </c>
+      <c r="O4" t="s">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="5" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>570</v>
+      </c>
+      <c r="B5" t="s">
+        <v>714</v>
+      </c>
+      <c r="C5" t="s">
+        <v>714</v>
+      </c>
+      <c r="D5" t="s">
+        <v>590</v>
+      </c>
+      <c r="E5" t="s">
+        <v>590</v>
+      </c>
+      <c r="F5" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="G5" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="H5" t="s">
+        <v>590</v>
+      </c>
+      <c r="K5" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="L5" t="s">
+        <v>590</v>
+      </c>
+      <c r="M5" t="s">
+        <v>590</v>
+      </c>
+      <c r="N5" t="s">
+        <v>714</v>
+      </c>
+      <c r="O5" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="6" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>575</v>
+      </c>
+      <c r="B6" t="s">
+        <v>805</v>
+      </c>
+      <c r="C6" t="s">
+        <v>805</v>
+      </c>
+      <c r="D6" t="s">
+        <v>850</v>
+      </c>
+      <c r="E6" t="s">
+        <v>850</v>
+      </c>
+      <c r="F6" t="s">
+        <v>834</v>
+      </c>
+      <c r="G6" t="s">
+        <v>834</v>
+      </c>
+      <c r="H6" t="s">
+        <v>850</v>
+      </c>
+      <c r="I6" t="s">
+        <v>864</v>
+      </c>
+      <c r="J6" t="s">
+        <v>864</v>
+      </c>
+      <c r="K6" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="L6" t="s">
+        <v>850</v>
+      </c>
+      <c r="M6" t="s">
+        <v>850</v>
+      </c>
+      <c r="N6" t="s">
+        <v>805</v>
+      </c>
+      <c r="O6" t="s">
+        <v>946</v>
+      </c>
+    </row>
+    <row r="7" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>576</v>
+      </c>
+      <c r="B7" t="s">
+        <v>947</v>
+      </c>
+      <c r="C7" t="s">
+        <v>947</v>
+      </c>
+      <c r="D7" t="s">
+        <v>948</v>
+      </c>
+      <c r="E7" t="s">
+        <v>948</v>
+      </c>
+      <c r="F7" s="30" t="s">
+        <v>949</v>
+      </c>
+      <c r="G7" s="30" t="s">
+        <v>950</v>
+      </c>
+      <c r="H7" t="s">
+        <v>951</v>
+      </c>
+      <c r="I7" t="s">
+        <v>952</v>
+      </c>
+      <c r="J7" t="s">
+        <v>952</v>
+      </c>
+      <c r="K7" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="L7" t="s">
+        <v>951</v>
+      </c>
+      <c r="M7" t="s">
+        <v>951</v>
+      </c>
+      <c r="N7" t="s">
+        <v>947</v>
+      </c>
+      <c r="O7" t="s">
+        <v>953</v>
+      </c>
+    </row>
+    <row r="9" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>577</v>
+      </c>
+      <c r="B9" t="s">
+        <v>745</v>
+      </c>
+      <c r="C9" t="s">
+        <v>745</v>
+      </c>
+      <c r="D9" t="s">
+        <v>745</v>
+      </c>
+      <c r="E9" t="s">
+        <v>745</v>
+      </c>
+      <c r="F9" t="s">
+        <v>745</v>
+      </c>
+      <c r="G9" t="s">
+        <v>745</v>
+      </c>
+      <c r="H9" t="s">
+        <v>745</v>
+      </c>
+      <c r="I9" t="s">
+        <v>745</v>
+      </c>
+      <c r="J9" t="s">
+        <v>745</v>
+      </c>
+      <c r="K9" t="s">
+        <v>745</v>
+      </c>
+      <c r="L9" t="s">
+        <v>745</v>
+      </c>
+      <c r="M9" t="s">
+        <v>745</v>
+      </c>
+      <c r="N9" t="s">
+        <v>745</v>
+      </c>
+      <c r="O9" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="10" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>578</v>
+      </c>
+      <c r="B10" t="s">
+        <v>767</v>
+      </c>
+      <c r="C10" t="s">
+        <v>767</v>
+      </c>
+      <c r="D10" t="s">
+        <v>954</v>
+      </c>
+      <c r="E10" t="s">
+        <v>954</v>
+      </c>
+      <c r="F10" t="s">
+        <v>955</v>
+      </c>
+      <c r="G10" t="s">
+        <v>955</v>
+      </c>
+      <c r="H10" t="s">
+        <v>767</v>
+      </c>
+      <c r="I10" t="s">
+        <v>957</v>
+      </c>
+      <c r="J10" t="s">
+        <v>957</v>
+      </c>
+      <c r="K10" s="31" t="s">
+        <v>956</v>
+      </c>
+      <c r="L10" t="s">
+        <v>767</v>
+      </c>
+      <c r="M10" t="s">
+        <v>767</v>
+      </c>
+      <c r="N10" t="s">
+        <v>767</v>
+      </c>
+      <c r="O10" t="s">
+        <v>958</v>
+      </c>
+    </row>
+    <row r="11" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>579</v>
+      </c>
+      <c r="B11" t="s">
+        <v>966</v>
+      </c>
+      <c r="C11" t="s">
+        <v>966</v>
+      </c>
+      <c r="D11" t="s">
+        <v>969</v>
+      </c>
+      <c r="E11" t="s">
+        <v>970</v>
+      </c>
+      <c r="F11" t="s">
+        <v>967</v>
+      </c>
+      <c r="G11" t="s">
+        <v>968</v>
+      </c>
+      <c r="H11" t="s">
+        <v>971</v>
+      </c>
+      <c r="I11" t="s">
+        <v>973</v>
+      </c>
+      <c r="J11" t="s">
+        <v>973</v>
+      </c>
+      <c r="K11" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="L11" t="s">
+        <v>971</v>
+      </c>
+      <c r="M11" t="s">
+        <v>971</v>
+      </c>
+      <c r="N11" t="s">
+        <v>966</v>
+      </c>
+      <c r="O11" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="12" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>580</v>
+      </c>
+      <c r="B12" t="s">
+        <v>722</v>
+      </c>
+      <c r="C12" t="s">
+        <v>722</v>
+      </c>
+      <c r="D12" t="s">
+        <v>959</v>
+      </c>
+      <c r="E12" t="s">
+        <v>960</v>
+      </c>
+      <c r="F12" t="s">
+        <v>961</v>
+      </c>
+      <c r="G12" t="s">
+        <v>962</v>
+      </c>
+      <c r="H12" t="s">
+        <v>963</v>
+      </c>
+      <c r="I12" t="s">
+        <v>964</v>
+      </c>
+      <c r="J12" t="s">
+        <v>964</v>
+      </c>
+      <c r="K12" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="L12" t="s">
+        <v>963</v>
+      </c>
+      <c r="M12" t="s">
+        <v>963</v>
+      </c>
+      <c r="N12" t="s">
+        <v>722</v>
+      </c>
+      <c r="O12" t="s">
+        <v>965</v>
+      </c>
+    </row>
+    <row r="13" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>581</v>
+      </c>
+      <c r="B13" t="s">
+        <v>989</v>
+      </c>
+      <c r="C13" t="s">
+        <v>989</v>
+      </c>
+      <c r="D13" t="s">
+        <v>990</v>
+      </c>
+      <c r="E13" t="s">
+        <v>990</v>
+      </c>
+      <c r="F13" t="s">
+        <v>629</v>
+      </c>
+      <c r="G13" t="s">
+        <v>629</v>
+      </c>
+      <c r="H13" t="s">
+        <v>989</v>
+      </c>
+      <c r="I13" t="s">
+        <v>857</v>
+      </c>
+      <c r="J13" t="s">
+        <v>857</v>
+      </c>
+      <c r="K13" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="L13" t="s">
+        <v>989</v>
+      </c>
+      <c r="M13" t="s">
+        <v>989</v>
+      </c>
+      <c r="N13" t="s">
+        <v>989</v>
+      </c>
+      <c r="O13" t="s">
+        <v>991</v>
+      </c>
+    </row>
+    <row r="14" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>582</v>
+      </c>
+      <c r="B14" t="s">
+        <v>974</v>
+      </c>
+      <c r="C14" t="s">
+        <v>974</v>
+      </c>
+      <c r="D14" t="s">
+        <v>872</v>
+      </c>
+      <c r="E14" t="s">
+        <v>872</v>
+      </c>
+      <c r="F14" t="s">
+        <v>621</v>
+      </c>
+      <c r="G14" t="s">
+        <v>621</v>
+      </c>
+      <c r="H14" t="s">
+        <v>974</v>
+      </c>
+      <c r="I14" t="s">
+        <v>976</v>
+      </c>
+      <c r="J14" t="s">
+        <v>976</v>
+      </c>
+      <c r="K14" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="L14" t="s">
+        <v>974</v>
+      </c>
+      <c r="M14" t="s">
+        <v>974</v>
+      </c>
+      <c r="N14" t="s">
+        <v>974</v>
+      </c>
+      <c r="O14" t="s">
+        <v>975</v>
+      </c>
+    </row>
+    <row r="15" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>583</v>
+      </c>
+      <c r="B15" t="s">
+        <v>977</v>
+      </c>
+      <c r="C15" t="s">
+        <v>977</v>
+      </c>
+      <c r="D15" t="s">
+        <v>978</v>
+      </c>
+      <c r="E15" t="s">
+        <v>978</v>
+      </c>
+      <c r="F15" t="s">
+        <v>979</v>
+      </c>
+      <c r="G15" t="s">
+        <v>980</v>
+      </c>
+      <c r="H15" t="s">
+        <v>977</v>
+      </c>
+      <c r="I15" t="s">
+        <v>861</v>
+      </c>
+      <c r="J15" t="s">
+        <v>861</v>
+      </c>
+      <c r="K15" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="L15" t="s">
+        <v>977</v>
+      </c>
+      <c r="M15" t="s">
+        <v>977</v>
+      </c>
+      <c r="N15" t="s">
+        <v>977</v>
+      </c>
+      <c r="O15" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="16" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>584</v>
+      </c>
+      <c r="B16" t="s">
+        <v>981</v>
+      </c>
+      <c r="C16" t="s">
+        <v>981</v>
+      </c>
+      <c r="D16" t="s">
+        <v>982</v>
+      </c>
+      <c r="E16" t="s">
+        <v>982</v>
+      </c>
+      <c r="F16" t="s">
+        <v>983</v>
+      </c>
+      <c r="G16" t="s">
+        <v>983</v>
+      </c>
+      <c r="H16" t="s">
+        <v>981</v>
+      </c>
+      <c r="I16" t="s">
+        <v>984</v>
+      </c>
+      <c r="J16" t="s">
+        <v>984</v>
+      </c>
+      <c r="K16" s="30" t="s">
+        <v>723</v>
+      </c>
+      <c r="L16" t="s">
+        <v>981</v>
+      </c>
+      <c r="M16" t="s">
+        <v>981</v>
+      </c>
+      <c r="N16" t="s">
+        <v>981</v>
+      </c>
+      <c r="O16" t="s">
+        <v>985</v>
+      </c>
+    </row>
+    <row r="20" spans="2:14" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B20" s="3" t="s">
+        <v>574</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>576</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>577</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>578</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>579</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>580</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>582</v>
+      </c>
+      <c r="M20" s="3" t="s">
+        <v>583</v>
+      </c>
+      <c r="N20" s="3" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="21" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B21" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>714</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>805</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>947</v>
+      </c>
+      <c r="G21" s="13" t="s">
+        <v>745</v>
+      </c>
+      <c r="H21" s="13" t="s">
+        <v>767</v>
+      </c>
+      <c r="I21" s="13" t="s">
+        <v>966</v>
+      </c>
+      <c r="J21" s="13" t="s">
+        <v>722</v>
+      </c>
+      <c r="K21" s="13" t="s">
+        <v>989</v>
+      </c>
+      <c r="L21" s="13" t="s">
+        <v>974</v>
+      </c>
+      <c r="M21" s="13" t="s">
+        <v>977</v>
+      </c>
+      <c r="N21" s="13" t="s">
+        <v>981</v>
+      </c>
+    </row>
+    <row r="22" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B22" s="13" t="s">
+        <v>586</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>590</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>850</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>948</v>
+      </c>
+      <c r="H22" s="13" t="s">
+        <v>603</v>
+      </c>
+      <c r="I22" s="13" t="s">
+        <v>969</v>
+      </c>
+      <c r="J22" s="13" t="s">
+        <v>959</v>
+      </c>
+      <c r="K22" s="13" t="s">
+        <v>990</v>
+      </c>
+      <c r="L22" s="13" t="s">
+        <v>872</v>
+      </c>
+      <c r="M22" s="13" t="s">
+        <v>978</v>
+      </c>
+      <c r="N22" s="13" t="s">
+        <v>982</v>
+      </c>
+    </row>
+    <row r="23" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B23" s="13" t="s">
+        <v>585</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>834</v>
+      </c>
+      <c r="E23" s="32" t="s">
+        <v>949</v>
+      </c>
+      <c r="F23" s="30"/>
+      <c r="H23" s="13" t="s">
+        <v>955</v>
+      </c>
+      <c r="I23" s="13" t="s">
+        <v>970</v>
+      </c>
+      <c r="J23" s="13" t="s">
+        <v>960</v>
+      </c>
+      <c r="K23" s="13" t="s">
+        <v>629</v>
+      </c>
+      <c r="L23" s="13" t="s">
+        <v>621</v>
+      </c>
+      <c r="M23" s="13" t="s">
+        <v>979</v>
+      </c>
+      <c r="N23" s="13" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B24" s="13" t="s">
+        <v>986</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>864</v>
+      </c>
+      <c r="E24" s="32" t="s">
+        <v>950</v>
+      </c>
+      <c r="H24" s="13" t="s">
+        <v>957</v>
+      </c>
+      <c r="I24" s="13" t="s">
+        <v>967</v>
+      </c>
+      <c r="J24" s="13" t="s">
+        <v>961</v>
+      </c>
+      <c r="K24" s="13" t="s">
+        <v>857</v>
+      </c>
+      <c r="L24" s="13" t="s">
+        <v>976</v>
+      </c>
+      <c r="M24" s="13" t="s">
+        <v>980</v>
+      </c>
+      <c r="N24" s="13" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="25" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B25" s="13" t="s">
+        <v>987</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>988</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>952</v>
+      </c>
+      <c r="H25" s="13" t="s">
+        <v>895</v>
+      </c>
+      <c r="I25" s="13" t="s">
+        <v>968</v>
+      </c>
+      <c r="J25" s="13" t="s">
+        <v>962</v>
+      </c>
+      <c r="K25" s="13" t="s">
+        <v>991</v>
+      </c>
+      <c r="L25" s="13" t="s">
+        <v>975</v>
+      </c>
+      <c r="M25" s="13" t="s">
+        <v>861</v>
+      </c>
+      <c r="N25" s="13" t="s">
+        <v>984</v>
+      </c>
+    </row>
+    <row r="26" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="D26" s="13" t="s">
+        <v>888</v>
+      </c>
+      <c r="E26" s="13" t="s">
+        <v>953</v>
+      </c>
+      <c r="H26" s="13" t="s">
+        <v>958</v>
+      </c>
+      <c r="I26" s="13" t="s">
+        <v>971</v>
+      </c>
+      <c r="J26" s="13" t="s">
+        <v>963</v>
+      </c>
+      <c r="M26" s="13" t="s">
+        <v>615</v>
+      </c>
+      <c r="N26" s="13" t="s">
+        <v>985</v>
+      </c>
+    </row>
+    <row r="27" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="I27" s="13" t="s">
+        <v>973</v>
+      </c>
+      <c r="J27" s="13" t="s">
+        <v>964</v>
+      </c>
+      <c r="M27" s="13"/>
+      <c r="N27" s="13"/>
+    </row>
+    <row r="28" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="I28" s="13" t="s">
+        <v>972</v>
+      </c>
+      <c r="J28" s="13" t="s">
+        <v>965</v>
+      </c>
+      <c r="M28" s="13"/>
+      <c r="N28" s="13"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>